<commit_message>
Save tag-corrected Uni-MMMU evaluation progress
</commit_message>
<xml_diff>
--- a/outputs/_eval/bagel-zebra-cot-lora-tagfix-actual/all_tasks_summary_bagel-zebra-cot-lora-tagfix-actual.xlsx
+++ b/outputs/_eval/bagel-zebra-cot-lora-tagfix-actual/all_tasks_summary_bagel-zebra-cot-lora-tagfix-actual.xlsx
@@ -485,6 +485,15 @@
       <c r="H2">
         <v>0.07857142857142857</v>
       </c>
+      <c r="I2">
+        <v>0.5286624203821656</v>
+      </c>
+      <c r="J2">
+        <v>0.3312101910828025</v>
+      </c>
+      <c r="K2">
+        <v>0.08917197452229299</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Save tag-corrected evaluation progress 2026-09-18T22:13:22Z
</commit_message>
<xml_diff>
--- a/outputs/_eval/bagel-zebra-cot-lora-tagfix-actual/all_tasks_summary_bagel-zebra-cot-lora-tagfix-actual.xlsx
+++ b/outputs/_eval/bagel-zebra-cot-lora-tagfix-actual/all_tasks_summary_bagel-zebra-cot-lora-tagfix-actual.xlsx
@@ -494,6 +494,15 @@
       <c r="K2">
         <v>0.08917197452229299</v>
       </c>
+      <c r="L2">
+        <v>0.145</v>
+      </c>
+      <c r="M2">
+        <v>0.01</v>
+      </c>
+      <c r="N2">
+        <v>0.01</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>